<commit_message>
chore(rbac): update RBAC configuration file
</commit_message>
<xml_diff>
--- a/db_storage/rbac.xlsx
+++ b/db_storage/rbac.xlsx
@@ -414,6 +414,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:A2"/>
   </ignoredErrors>
@@ -494,7 +495,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
+      <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="str">
@@ -520,7 +521,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
+      <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="str">
@@ -546,7 +547,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
+      <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="str">
@@ -572,7 +573,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
+      <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="str">
@@ -598,7 +599,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
+      <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="str">
@@ -624,7 +625,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
+      <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="str">
@@ -650,7 +651,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="str">
+      <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="str">
@@ -676,7 +677,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="str">
+      <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="str">
@@ -702,7 +703,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="str">
+      <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="str">
@@ -728,7 +729,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="str">
+      <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="str">
@@ -754,7 +755,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="str">
+      <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="str">
@@ -780,7 +781,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="str">
+      <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="str">
@@ -831,7 +832,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
+      <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="str">
@@ -845,7 +846,7 @@
       </c>
     </row>
     <row r="3" xml:space="preserve">
-      <c r="A3" t="str">
+      <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="str" xml:space="preserve">
@@ -860,6 +861,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
   </ignoredErrors>
@@ -868,7 +870,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -897,7 +899,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
+      <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="str">
@@ -919,11 +921,11 @@
         <v>2026-04-29T13:28:28.588Z</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-05-10T14:50:24.231Z</v>
+        <v>2026-05-04T08:59:46.843Z</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
+      <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="str">
@@ -946,42 +948,238 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>3</v>
+      <c r="A4">
+        <v>5</v>
       </c>
       <c r="B4" t="str">
-        <v>Ravindra Reddy</v>
+        <v>Ravi Boss</v>
       </c>
       <c r="C4" t="str">
-        <v>ravindramprelive</v>
+        <v xml:space="preserve">ravindra.munnangi@arrise.com  </v>
       </c>
       <c r="D4" t="str">
-        <v>ADMIN</v>
+        <v>ADMIN,USER</v>
+      </c>
+      <c r="F4" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-05-05T16:15:36.777Z</v>
+        <v>2026-05-08T13:19:39.847Z</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-05-05T16:15:36.777Z</v>
+        <v>2026-05-08T13:19:39.847Z</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
-        <v>4</v>
+      <c r="A5">
+        <v>6</v>
       </c>
       <c r="B5" t="str">
-        <v>Ravindra reddy</v>
+        <v xml:space="preserve">Nanda </v>
       </c>
       <c r="C5" t="str">
-        <v>ravindra.munnangi@arrise.com</v>
+        <v>nandagopala.chilukuri@arrise.com</v>
       </c>
       <c r="D5" t="str">
-        <v>ADMIN</v>
+        <v>USER</v>
+      </c>
+      <c r="F5" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2026-05-10T21:06:00.086Z</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2026-05-10T21:06:13.701Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>7</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Gowtham</v>
+      </c>
+      <c r="C6" t="str">
+        <v>gowtham.ramineni@arrise.com</v>
+      </c>
+      <c r="D6" t="str">
+        <v>USER</v>
+      </c>
+      <c r="F6" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-05-10T21:07:20.507Z</v>
+      </c>
+      <c r="H6" t="str">
+        <v>2026-05-10T21:07:20.507Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>8</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Bala</v>
+      </c>
+      <c r="C7" t="str">
+        <v>balasaheb.tathe@arrise.com</v>
+      </c>
+      <c r="D7" t="str">
+        <v>USER</v>
+      </c>
+      <c r="F7" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2026-05-10T21:07:57.160Z</v>
+      </c>
+      <c r="H7" t="str">
+        <v>2026-05-10T21:07:57.160Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>9</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Raja</v>
+      </c>
+      <c r="C8" t="str">
+        <v>ravipati.raja@arrise.com</v>
+      </c>
+      <c r="D8" t="str">
+        <v>USER</v>
+      </c>
+      <c r="F8" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+      </c>
+      <c r="G8" t="str">
+        <v>2026-05-10T21:08:52.951Z</v>
+      </c>
+      <c r="H8" t="str">
+        <v>2026-05-10T21:10:15.222Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>10</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Uday</v>
+      </c>
+      <c r="C9" t="str">
+        <v>uday.mali@arrise.com</v>
+      </c>
+      <c r="D9" t="str">
+        <v>USER</v>
+      </c>
+      <c r="F9" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+      </c>
+      <c r="G9" t="str">
+        <v>2026-05-10T21:10:00.306Z</v>
+      </c>
+      <c r="H9" t="str">
+        <v>2026-05-10T21:10:00.306Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>11</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Shirish Jaiswal</v>
+      </c>
+      <c r="C10" t="str">
+        <v>shirish.jaiswal@arrise.com</v>
+      </c>
+      <c r="D10" t="str">
+        <v>ADMIN,USER</v>
+      </c>
+      <c r="F10" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2026-05-10T21:13:06.791Z</v>
+      </c>
+      <c r="H10" t="str">
+        <v>2026-05-10T21:13:06.791Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>12</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Gaurav Khandelwal</v>
+      </c>
+      <c r="C11" t="str">
+        <v>gaurav.khandelwal@arrise.com</v>
+      </c>
+      <c r="D11" t="str">
+        <v>USER,ADMIN</v>
+      </c>
+      <c r="F11" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+      </c>
+      <c r="G11" t="str">
+        <v>2026-05-10T21:14:01.370Z</v>
+      </c>
+      <c r="H11" t="str">
+        <v>2026-05-10T21:14:01.370Z</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>13</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Mallikarjun Reddy V</v>
+      </c>
+      <c r="C12" t="str">
+        <v>mallikarjun.reddy@arrise.com</v>
+      </c>
+      <c r="D12" t="str">
+        <v>ADMIN,USER</v>
+      </c>
+      <c r="F12" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+      </c>
+      <c r="G12" t="str">
+        <v>2026-05-10T21:14:50.906Z</v>
+      </c>
+      <c r="H12" t="str">
+        <v>2026-05-10T21:14:50.906Z</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>14</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Siva Tandam</v>
+      </c>
+      <c r="C13" t="str">
+        <v>siva.tandam@arrise.com</v>
+      </c>
+      <c r="D13" t="str">
+        <v>ADMIN,USER</v>
+      </c>
+      <c r="F13" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+      </c>
+      <c r="G13" t="str">
+        <v>2026-05-10T21:15:38.156Z</v>
+      </c>
+      <c r="H13" t="str">
+        <v>2026-05-10T21:15:38.156Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor(proxy): update F_DOMAIN usage and clean up console logs
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/db_storage/rbac.xlsx
+++ b/db_storage/rbac.xlsx
@@ -870,7 +870,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1177,9 +1177,32 @@
         <v>2026-05-10T21:15:38.156Z</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14">
+        <v>15</v>
+      </c>
+      <c r="B14" t="str">
+        <v>ravindramprelive</v>
+      </c>
+      <c r="C14" t="str">
+        <v>ravindramprelive</v>
+      </c>
+      <c r="D14" t="str">
+        <v>USER</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v>2026-05-10T22:01:00.676Z</v>
+      </c>
+      <c r="H14" t="str">
+        <v>2026-05-10T22:01:15.187Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor game metadata handling and add new game plugins
- Updated Tabs component styling for better layout.
- Removed obsolete game-handlers.ts and integrated game logic into individual plugins.
- Introduced new game plugins for Baccarat, Crash Game, Game Show, Roulette, Sweet Bonanza, and Treasure Island.
- Enhanced game type detection to include "treasure-island".
- Improved column resizing logic in LogTable component.
- Updated RoundDetailsProvider to allow more round and game IDs.
- Refined styles for various game results in styleMap.
- Added utility functions for label building and data normalization.

Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/db_storage/rbac.xlsx
+++ b/db_storage/rbac.xlsx
@@ -870,7 +870,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H22"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -909,19 +909,19 @@
         <v>rajani.rachakonda@arrise.com</v>
       </c>
       <c r="D2" t="str">
-        <v>ADMIN</v>
+        <v>ADMIN,USER</v>
       </c>
       <c r="E2" t="str">
         <v>U2FsdGVkX18286Us/KPbmUYKh7Kj/JAgrjWI5rcex90=</v>
       </c>
       <c r="F2" t="str">
-        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
       </c>
       <c r="G2" t="str">
         <v>2026-04-29T13:28:28.588Z</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-05-04T08:59:46.843Z</v>
+        <v>2026-05-10T22:46:30.891Z</v>
       </c>
     </row>
     <row r="3">
@@ -937,6 +937,9 @@
       <c r="D3" t="str">
         <v>ADMIN,USER</v>
       </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
       <c r="F3" t="str">
         <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
       </c>
@@ -944,7 +947,7 @@
         <v>2026-05-05T12:36:15.150Z</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-05-05T12:36:15.150Z</v>
+        <v>2026-05-11T07:41:00.437Z</v>
       </c>
     </row>
     <row r="4">
@@ -961,13 +964,13 @@
         <v>ADMIN,USER</v>
       </c>
       <c r="F4" t="str">
-        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
       </c>
       <c r="G4" t="str">
         <v>2026-05-08T13:19:39.847Z</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-05-08T13:19:39.847Z</v>
+        <v>2026-05-10T22:44:35.455Z</v>
       </c>
     </row>
     <row r="5">
@@ -984,13 +987,13 @@
         <v>USER</v>
       </c>
       <c r="F5" t="str">
-        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
       </c>
       <c r="G5" t="str">
         <v>2026-05-10T21:06:00.086Z</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-05-10T21:06:13.701Z</v>
+        <v>2026-05-10T22:44:40.249Z</v>
       </c>
     </row>
     <row r="6">
@@ -1007,13 +1010,13 @@
         <v>USER</v>
       </c>
       <c r="F6" t="str">
-        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
       </c>
       <c r="G6" t="str">
         <v>2026-05-10T21:07:20.507Z</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-05-10T21:07:20.507Z</v>
+        <v>2026-05-10T22:45:50.445Z</v>
       </c>
     </row>
     <row r="7">
@@ -1029,6 +1032,9 @@
       <c r="D7" t="str">
         <v>USER</v>
       </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
       <c r="F7" t="str">
         <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
       </c>
@@ -1036,7 +1042,7 @@
         <v>2026-05-10T21:07:57.160Z</v>
       </c>
       <c r="H7" t="str">
-        <v>2026-05-10T21:07:57.160Z</v>
+        <v>2026-05-11T05:01:30.046Z</v>
       </c>
     </row>
     <row r="8">
@@ -1053,13 +1059,13 @@
         <v>USER</v>
       </c>
       <c r="F8" t="str">
-        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
       </c>
       <c r="G8" t="str">
         <v>2026-05-10T21:08:52.951Z</v>
       </c>
       <c r="H8" t="str">
-        <v>2026-05-10T21:10:15.222Z</v>
+        <v>2026-05-10T22:45:45.333Z</v>
       </c>
     </row>
     <row r="9">
@@ -1076,13 +1082,13 @@
         <v>USER</v>
       </c>
       <c r="F9" t="str">
-        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
       </c>
       <c r="G9" t="str">
         <v>2026-05-10T21:10:00.306Z</v>
       </c>
       <c r="H9" t="str">
-        <v>2026-05-10T21:10:00.306Z</v>
+        <v>2026-05-10T22:45:40.380Z</v>
       </c>
     </row>
     <row r="10">
@@ -1098,6 +1104,9 @@
       <c r="D10" t="str">
         <v>ADMIN,USER</v>
       </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
       <c r="F10" t="str">
         <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
       </c>
@@ -1105,7 +1114,7 @@
         <v>2026-05-10T21:13:06.791Z</v>
       </c>
       <c r="H10" t="str">
-        <v>2026-05-10T21:13:06.791Z</v>
+        <v>2026-05-11T03:36:55.550Z</v>
       </c>
     </row>
     <row r="11">
@@ -1122,13 +1131,13 @@
         <v>USER,ADMIN</v>
       </c>
       <c r="F11" t="str">
-        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
       </c>
       <c r="G11" t="str">
         <v>2026-05-10T21:14:01.370Z</v>
       </c>
       <c r="H11" t="str">
-        <v>2026-05-10T21:14:01.370Z</v>
+        <v>2026-05-10T22:45:13.123Z</v>
       </c>
     </row>
     <row r="12">
@@ -1145,13 +1154,13 @@
         <v>ADMIN,USER</v>
       </c>
       <c r="F12" t="str">
-        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
       </c>
       <c r="G12" t="str">
         <v>2026-05-10T21:14:50.906Z</v>
       </c>
       <c r="H12" t="str">
-        <v>2026-05-10T21:14:50.906Z</v>
+        <v>2026-05-10T22:45:06.777Z</v>
       </c>
     </row>
     <row r="13">
@@ -1168,41 +1177,231 @@
         <v>ADMIN,USER</v>
       </c>
       <c r="F13" t="str">
-        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
       </c>
       <c r="G13" t="str">
         <v>2026-05-10T21:15:38.156Z</v>
       </c>
       <c r="H13" t="str">
-        <v>2026-05-10T21:15:38.156Z</v>
+        <v>2026-05-10T22:45:02.049Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B14" t="str">
-        <v>ravindramprelive</v>
+        <v>Gaurav Khandelwal</v>
       </c>
       <c r="C14" t="str">
-        <v>ravindramprelive</v>
+        <v>gauravlive</v>
       </c>
       <c r="D14" t="str">
+        <v>ADMIN,USER</v>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+      </c>
+      <c r="G14" t="str">
+        <v>2026-05-11T05:24:50.903Z</v>
+      </c>
+      <c r="H14" t="str">
+        <v>2026-05-11T05:25:25.605Z</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>17</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Ramesh</v>
+      </c>
+      <c r="C15" t="str">
+        <v>ramesh.komakula@arrise.com</v>
+      </c>
+      <c r="D15" t="str">
         <v>USER</v>
       </c>
-      <c r="F14" t="str">
+      <c r="F15" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
+      </c>
+      <c r="G15" t="str">
+        <v>2026-05-11T07:38:58.963Z</v>
+      </c>
+      <c r="H15" t="str">
+        <v>2026-05-11T07:45:09.741Z</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>18</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Amireddy</v>
+      </c>
+      <c r="C16" t="str">
+        <v>ami.reddy@arrise.com</v>
+      </c>
+      <c r="D16" t="str">
+        <v>USER</v>
+      </c>
+      <c r="F16" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
+      </c>
+      <c r="G16" t="str">
+        <v>2026-05-11T07:42:15.041Z</v>
+      </c>
+      <c r="H16" t="str">
+        <v>2026-05-11T07:45:14.246Z</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>19</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Yasasvi</v>
+      </c>
+      <c r="C17" t="str">
+        <v>yasasvidurga.g@arrise.com</v>
+      </c>
+      <c r="D17" t="str">
+        <v>USER</v>
+      </c>
+      <c r="F17" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
+      </c>
+      <c r="G17" t="str">
+        <v>2026-05-11T07:43:13.496Z</v>
+      </c>
+      <c r="H17" t="str">
+        <v>2026-05-11T07:45:18.180Z</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>20</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Vigneshwari</v>
+      </c>
+      <c r="C18" t="str">
+        <v>vigneshwarireddy.m@arrise.com</v>
+      </c>
+      <c r="D18" t="str">
+        <v>USER</v>
+      </c>
+      <c r="F18" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
+      </c>
+      <c r="G18" t="str">
+        <v>2026-05-11T07:44:05.061Z</v>
+      </c>
+      <c r="H18" t="str">
+        <v>2026-05-11T07:45:24.332Z</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>21</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Dishil</v>
+      </c>
+      <c r="C19" t="str">
+        <v>dishil.p@arrise.com</v>
+      </c>
+      <c r="D19" t="str">
+        <v>USER</v>
+      </c>
+      <c r="E19" t="str">
         <v/>
       </c>
-      <c r="G14" t="str">
-        <v>2026-05-10T22:01:00.676Z</v>
-      </c>
-      <c r="H14" t="str">
-        <v>2026-05-10T22:01:15.187Z</v>
+      <c r="F19" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+      </c>
+      <c r="G19" t="str">
+        <v>2026-05-11T07:44:25.215Z</v>
+      </c>
+      <c r="H19" t="str">
+        <v>2026-05-11T09:19:32.932Z</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>22</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Raghavendra</v>
+      </c>
+      <c r="C20" t="str">
+        <v>raghavendra.konda@arrise.com</v>
+      </c>
+      <c r="D20" t="str">
+        <v>USER</v>
+      </c>
+      <c r="F20" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
+      </c>
+      <c r="G20" t="str">
+        <v>2026-05-11T07:44:58.955Z</v>
+      </c>
+      <c r="H20" t="str">
+        <v>2026-05-11T07:45:37.803Z</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>23</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Siva</v>
+      </c>
+      <c r="C21" t="str">
+        <v>sivatandam</v>
+      </c>
+      <c r="D21" t="str">
+        <v>ADMIN,USER</v>
+      </c>
+      <c r="F21" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
+      </c>
+      <c r="G21" t="str">
+        <v>2026-05-11T09:05:01.748Z</v>
+      </c>
+      <c r="H21" t="str">
+        <v>2026-05-11T11:31:41.750Z</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>24</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Tiago Moura</v>
+      </c>
+      <c r="C22" t="str">
+        <v>tiago.moura@arrise.com</v>
+      </c>
+      <c r="D22" t="str">
+        <v>USER</v>
+      </c>
+      <c r="F22" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
+      </c>
+      <c r="G22" t="str">
+        <v>2026-05-11T11:31:22.511Z</v>
+      </c>
+      <c r="H22" t="str">
+        <v>2026-05-11T11:34:26.047Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add audit logs UI
</commit_message>
<xml_diff>
--- a/db_storage/rbac.xlsx
+++ b/db_storage/rbac.xlsx
@@ -466,7 +466,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -806,9 +806,35 @@
         <v>2026-05-02T08:01:25.792Z</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Auditlog</v>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v>/audit-logs</v>
+      </c>
+      <c r="E14" t="str">
+        <v>ADMIN</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Administration</v>
+      </c>
+      <c r="G14" t="str">
+        <v>2026-05-13T17:40:18.760Z</v>
+      </c>
+      <c r="H14" t="str">
+        <v>2026-05-13T18:44:33.152Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -870,7 +896,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1399,9 +1425,32 @@
         <v>2026-05-11T11:34:26.047Z</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23">
+        <v>25</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Ravindra</v>
+      </c>
+      <c r="C23" t="str">
+        <v>ravindramlive</v>
+      </c>
+      <c r="D23" t="str">
+        <v>USER</v>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v>2026-05-13T20:07:01.943Z</v>
+      </c>
+      <c r="H23" t="str">
+        <v>2026-05-13T20:07:01.943Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H23"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: enhance text editor toolbar with log functionality and improve UI components
- Added LogTogglePlugin to the text editor toolbar for inserting logs.
- Introduced log command and utility functions for handling log data.
- Updated Toolbar component to conditionally render log toggle.
- Enhanced game result sheets with ResultSheetHeaderBlock for displaying game details.
- Improved styling and structure of various game metadata components.
- Refactored usePlayerBetHistory hook to handle concurrency in fetching player bet history.
- Updated schemas in types for better data validation and trimming.
- Made adjustments to resolution editor for improved layout and functionality.

Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/db_storage/rbac.xlsx
+++ b/db_storage/rbac.xlsx
@@ -823,13 +823,13 @@
         <v>ADMIN</v>
       </c>
       <c r="F14" t="str">
-        <v>Tools</v>
+        <v>TOOLS</v>
       </c>
       <c r="G14" t="str">
         <v>2026-05-14T11:07:13.355Z</v>
       </c>
       <c r="H14" t="str">
-        <v>2026-05-14T11:07:13.355Z</v>
+        <v>2026-05-14T11:56:03.157Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add Blackjack result renderer and transformer for game results
- Implemented `BlackjackResultRenderer` to display game results in a structured table format.
- Created `blackjack-transformer` to transform raw game data into the format required by the renderer.
- Established a game result registry to manage different game types, including Blackjack and Baccarat.
- Introduced a universal game configuration type to support mixed game lists.
- Added UI components for Freshdesk ticket management, including message cards, sections, and a workspace for ticket interactions.
- Developed API functions for adding notes to Freshdesk tickets and retrieving decrypted API keys.
- Enhanced message body formatting for links in Freshdesk messages.
</commit_message>
<xml_diff>
--- a/db_storage/rbac.xlsx
+++ b/db_storage/rbac.xlsx
@@ -922,7 +922,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H29"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1048,7 +1048,7 @@
         <v>2026-05-10T21:06:00.086Z</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-05-10T22:44:40.249Z</v>
+        <v>2026-06-03T09:24:44.347Z</v>
       </c>
     </row>
     <row r="6">
@@ -1578,9 +1578,55 @@
         <v>2026-05-29T13:04:02.299Z</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28">
+        <v>30</v>
+      </c>
+      <c r="B28" t="str">
+        <v>flores</v>
+      </c>
+      <c r="C28" t="str">
+        <v>flores</v>
+      </c>
+      <c r="D28" t="str">
+        <v>USER</v>
+      </c>
+      <c r="F28" t="str">
+        <v>{"doYouKnow":{"title":"doyouknow","on":true},"qna":{"title":"qna","on":true}}</v>
+      </c>
+      <c r="G28" t="str">
+        <v>2026-06-03T09:24:38.136Z</v>
+      </c>
+      <c r="H28" t="str">
+        <v>2026-06-03T09:24:56.222Z</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>31</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Ravindra-prelive</v>
+      </c>
+      <c r="C29" t="str">
+        <v>ravindramprelive</v>
+      </c>
+      <c r="D29" t="str">
+        <v>ADMIN,USER</v>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v>2026-06-03T10:06:34.966Z</v>
+      </c>
+      <c r="H29" t="str">
+        <v>2026-06-03T10:06:34.966Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H29"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: remove console.log statements for cleaner code
</commit_message>
<xml_diff>
--- a/db_storage/rbac.xlsx
+++ b/db_storage/rbac.xlsx
@@ -1166,7 +1166,7 @@
         <v>ADMIN,USER</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>U2FsdGVkX19PlyUmw3rHKvYtH0KrO5XKeyHbW2roMdnmy2rcgAYnzwvTnASx6l5d</v>
       </c>
       <c r="F10" t="str">
         <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
@@ -1175,7 +1175,7 @@
         <v>2026-05-10T21:13:06.791Z</v>
       </c>
       <c r="H10" t="str">
-        <v>2026-05-11T03:36:55.550Z</v>
+        <v>2026-06-05T20:38:58.520Z</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
refactor: improve game result components by extracting formatting functions and updating UI logic
</commit_message>
<xml_diff>
--- a/db_storage/rbac.xlsx
+++ b/db_storage/rbac.xlsx
@@ -1169,13 +1169,13 @@
         <v>U2FsdGVkX19PlyUmw3rHKvYtH0KrO5XKeyHbW2roMdnmy2rcgAYnzwvTnASx6l5d</v>
       </c>
       <c r="F10" t="str">
-        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false}}</v>
+        <v>{"doYouKnow":{"title":"doyouknow","on":false},"qna":{"title":"qna","on":false},"defaultCountry":"India"}</v>
       </c>
       <c r="G10" t="str">
         <v>2026-05-10T21:13:06.791Z</v>
       </c>
       <c r="H10" t="str">
-        <v>2026-06-05T20:38:58.520Z</v>
+        <v>2026-06-07T18:27:58.020Z</v>
       </c>
     </row>
     <row r="11">

</xml_diff>